<commit_message>
Fixtures: vary messy_qualtrics Q10 open-ended responses (25-comment pool, blanks, quotes, newlines, email lookalikes)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P3D4BbGJecLYmxuzn4n6UZ
</commit_message>
<xml_diff>
--- a/fixtures/practice/messy_qualtrics/messy.xlsx
+++ b/fixtures/practice/messy_qualtrics/messy.xlsx
@@ -1093,8 +1093,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>More practice problems would help, please add some.</t>
         </is>
       </c>
       <c r="AH4" t="n">
@@ -1226,8 +1225,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>It was fine. Nothing special, nothing terrible.</t>
         </is>
       </c>
       <c r="AH5" t="n">
@@ -1363,8 +1361,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Study groups were helpful, especially before quizzes.</t>
         </is>
       </c>
       <c r="AH6" t="n">
@@ -1500,8 +1497,7 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH7" t="n">
@@ -1633,8 +1629,7 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH8" t="n">
@@ -1766,8 +1761,8 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH9" t="n">
@@ -2036,8 +2031,7 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Best math teacher I've had, would take another class with them.</t>
         </is>
       </c>
       <c r="AH11" t="n">
@@ -2169,8 +2163,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>It was fine. Nothing special, nothing terrible.</t>
         </is>
       </c>
       <c r="AH12" t="n">
@@ -2302,8 +2295,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I'd recommend adding more review sessions, practice quizzes, and examples.</t>
         </is>
       </c>
       <c r="AH13" t="n">
@@ -2439,8 +2431,7 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH14" t="n">
@@ -2572,8 +2563,7 @@
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH15" t="n">
@@ -2705,8 +2695,7 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH16" t="n">
@@ -2840,12 +2829,7 @@
           <t>You can reach me at student85@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG17" t="inlineStr"/>
       <c r="AH17" t="n">
         <v>80</v>
       </c>
@@ -2977,12 +2961,7 @@
           <t>You can reach me at student81@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="n">
         <v>82</v>
       </c>
@@ -3116,8 +3095,7 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Feel free to reach out at abarnes@school.edu with any follow-up questions.</t>
         </is>
       </c>
       <c r="AH19" t="n">
@@ -3253,8 +3231,7 @@
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Study groups were helpful, especially before quizzes.</t>
         </is>
       </c>
       <c r="AH20" t="n">
@@ -3386,8 +3363,8 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH21" t="n">
@@ -3517,12 +3494,7 @@
           <t>You can reach me at student74@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="n">
         <v>68</v>
       </c>
@@ -3785,8 +3757,7 @@
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH24" t="n">
@@ -3918,8 +3889,7 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH25" t="n">
@@ -4049,12 +4019,7 @@
           <t>You can reach me at student19@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="n">
         <v>73</v>
       </c>
@@ -4184,8 +4149,7 @@
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>More practice problems would help, please add some.</t>
         </is>
       </c>
       <c r="AH27" t="n">
@@ -4317,8 +4281,7 @@
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Loved the group projects, hated the exams.</t>
         </is>
       </c>
       <c r="AH28" t="n">
@@ -4450,8 +4413,7 @@
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The pacing was uneven: too slow in week 1, too fast by week 10.</t>
         </is>
       </c>
       <c r="AH29" t="n">
@@ -4587,8 +4549,7 @@
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH30" t="n">
@@ -4720,8 +4681,7 @@
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Great class overall, thanks for a good semester.</t>
         </is>
       </c>
       <c r="AH31" t="n">
@@ -4857,8 +4817,7 @@
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I struggled with the pace at first, but it got better.</t>
         </is>
       </c>
       <c r="AH32" t="n">
@@ -4990,8 +4949,7 @@
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Honestly, I think this was one of my favorite math classes.</t>
         </is>
       </c>
       <c r="AH33" t="n">
@@ -5123,8 +5081,7 @@
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Feel free to reach out at abarnes@school.edu with any follow-up questions.</t>
         </is>
       </c>
       <c r="AH34" t="n">
@@ -5254,12 +5211,7 @@
           <t>You can reach me at student89@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG35" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG35" t="inlineStr"/>
       <c r="AH35" t="n">
         <v>71</v>
       </c>
@@ -5389,8 +5341,7 @@
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH36" t="n">
@@ -5522,8 +5473,7 @@
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH37" t="n">
@@ -5653,12 +5603,7 @@
           <t>You can reach me at student69@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG38" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="n">
         <v>70</v>
       </c>
@@ -5788,8 +5733,7 @@
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH39" t="n">
@@ -5921,8 +5865,7 @@
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The pacing was uneven: too slow in week 1, too fast by week 10.</t>
         </is>
       </c>
       <c r="AH40" t="n">
@@ -6054,8 +5997,7 @@
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Great class overall, thanks for a good semester.</t>
         </is>
       </c>
       <c r="AH41" t="n">
@@ -6187,8 +6129,7 @@
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH42" t="n">
@@ -6318,12 +6259,7 @@
           <t>You can reach me at student48@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG43" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="n">
         <v>68</v>
       </c>
@@ -6453,8 +6389,7 @@
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>More practice problems would help, please add some.</t>
         </is>
       </c>
       <c r="AH44" t="n">
@@ -6586,8 +6521,7 @@
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The pacing was uneven: too slow in week 1, too fast by week 10.</t>
         </is>
       </c>
       <c r="AH45" t="n">
@@ -6719,8 +6653,7 @@
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I'd recommend adding more review sessions, practice quizzes, and examples.</t>
         </is>
       </c>
       <c r="AH46" t="n">
@@ -6852,8 +6785,7 @@
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The "flipped classroom" approach didn't work for me.</t>
         </is>
       </c>
       <c r="AH47" t="n">
@@ -6985,8 +6917,7 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The "flipped classroom" approach didn't work for me.</t>
         </is>
       </c>
       <c r="AH48" t="n">
@@ -7118,8 +7049,7 @@
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH49" t="n">
@@ -7251,8 +7181,7 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The pacing was uneven: too slow in week 1, too fast by week 10.</t>
         </is>
       </c>
       <c r="AH50" t="n">
@@ -7388,8 +7317,7 @@
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I'd recommend adding more review sessions, practice quizzes, and examples.</t>
         </is>
       </c>
       <c r="AH51" t="n">
@@ -7521,8 +7449,7 @@
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH52" t="n">
@@ -7654,8 +7581,7 @@
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Loved the group projects, hated the exams.</t>
         </is>
       </c>
       <c r="AH53" t="n">
@@ -7787,8 +7713,7 @@
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH54" t="n">
@@ -7920,8 +7845,7 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Great class overall, thanks for a good semester.</t>
         </is>
       </c>
       <c r="AH55" t="n">
@@ -8053,8 +7977,7 @@
       </c>
       <c r="AG56" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH56" t="n">
@@ -8186,8 +8109,7 @@
       </c>
       <c r="AG57" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Honestly, I think this was one of my favorite math classes.</t>
         </is>
       </c>
       <c r="AH57" t="n">
@@ -8323,8 +8245,7 @@
       </c>
       <c r="AG58" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH58" t="n">
@@ -8456,8 +8377,7 @@
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Feel free to reach out at abarnes@school.edu with any follow-up questions.</t>
         </is>
       </c>
       <c r="AH59" t="n">
@@ -8589,8 +8509,8 @@
       </c>
       <c r="AG60" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH60" t="n">
@@ -8726,8 +8646,8 @@
       </c>
       <c r="AG61" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH61" t="n">
@@ -8859,8 +8779,7 @@
       </c>
       <c r="AG62" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>It was fine. Nothing special, nothing terrible.</t>
         </is>
       </c>
       <c r="AH62" t="n">
@@ -8992,8 +8911,7 @@
       </c>
       <c r="AG63" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>If you have questions about the final, email me at jsmith@school.edu.</t>
         </is>
       </c>
       <c r="AH63" t="n">
@@ -9129,8 +9047,7 @@
       </c>
       <c r="AG64" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>If you have questions about the final, email me at jsmith@school.edu.</t>
         </is>
       </c>
       <c r="AH64" t="n">
@@ -9262,8 +9179,7 @@
       </c>
       <c r="AG65" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH65" t="n">
@@ -9395,8 +9311,7 @@
       </c>
       <c r="AG66" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Great class overall, thanks for a good semester.</t>
         </is>
       </c>
       <c r="AH66" t="n">
@@ -9528,8 +9443,7 @@
       </c>
       <c r="AG67" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Feel free to reach out at abarnes@school.edu with any follow-up questions.</t>
         </is>
       </c>
       <c r="AH67" t="n">
@@ -9661,8 +9575,7 @@
       </c>
       <c r="AG68" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The online videos were confusing, but the textbook helped.</t>
         </is>
       </c>
       <c r="AH68" t="n">
@@ -9798,8 +9711,7 @@
       </c>
       <c r="AG69" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The online videos were confusing, but the textbook helped.</t>
         </is>
       </c>
       <c r="AH69" t="n">
@@ -9931,8 +9843,7 @@
       </c>
       <c r="AG70" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH70" t="n">
@@ -10068,8 +9979,7 @@
       </c>
       <c r="AG71" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The "flipped classroom" approach didn't work for me.</t>
         </is>
       </c>
       <c r="AH71" t="n">
@@ -10201,8 +10111,8 @@
       </c>
       <c r="AG72" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH72" t="n">
@@ -10334,8 +10244,7 @@
       </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I struggled with the pace at first, but it got better.</t>
         </is>
       </c>
       <c r="AH73" t="n">
@@ -10598,12 +10507,7 @@
           <t>You can reach me at student35@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG75" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG75" t="inlineStr"/>
       <c r="AH75" t="n">
         <v>82</v>
       </c>
@@ -10733,8 +10637,7 @@
       </c>
       <c r="AG76" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH76" t="n">
@@ -10864,12 +10767,7 @@
           <t>You can reach me at student54@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG77" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG77" t="inlineStr"/>
       <c r="AH77" t="n">
         <v>94</v>
       </c>
@@ -10999,8 +10897,7 @@
       </c>
       <c r="AG78" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH78" t="n">
@@ -11134,12 +11031,7 @@
           <t>You can reach me at student98@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG79" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG79" t="inlineStr"/>
       <c r="AH79" t="n">
         <v>89</v>
       </c>
@@ -11273,8 +11165,7 @@
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>It was fine. Nothing special, nothing terrible.</t>
         </is>
       </c>
       <c r="AH80" t="n">
@@ -11541,12 +11432,7 @@
           <t>You can reach me at student25@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG82" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG82" t="inlineStr"/>
       <c r="AH82" t="n">
         <v>81</v>
       </c>
@@ -11678,12 +11564,7 @@
           <t>You can reach me at student63@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG83" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG83" t="inlineStr"/>
       <c r="AH83" t="n">
         <v>94</v>
       </c>
@@ -11813,8 +11694,7 @@
       </c>
       <c r="AG84" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH84" t="n">
@@ -12077,12 +11957,7 @@
           <t>You can reach me at student80@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG86" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG86" t="inlineStr"/>
       <c r="AH86" t="n">
         <v>79</v>
       </c>
@@ -12212,8 +12087,7 @@
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I'd recommend adding more review sessions, practice quizzes, and examples.</t>
         </is>
       </c>
       <c r="AH87" t="n">
@@ -12343,12 +12217,7 @@
           <t>You can reach me at student109@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG88" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG88" t="inlineStr"/>
       <c r="AH88" t="n">
         <v>89</v>
       </c>
@@ -12478,8 +12347,7 @@
       </c>
       <c r="AG89" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH89" t="n">
@@ -12611,8 +12479,7 @@
       </c>
       <c r="AG90" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The online videos were confusing, but the textbook helped.</t>
         </is>
       </c>
       <c r="AH90" t="n">
@@ -12742,12 +12609,7 @@
           <t>You can reach me at student91@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG91" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG91" t="inlineStr"/>
       <c r="AH91" t="n">
         <v>63</v>
       </c>
@@ -12877,8 +12739,7 @@
       </c>
       <c r="AG92" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I'd recommend adding more review sessions, practice quizzes, and examples.</t>
         </is>
       </c>
       <c r="AH92" t="n">
@@ -13014,8 +12875,7 @@
       </c>
       <c r="AG93" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Study groups were helpful, especially before quizzes.</t>
         </is>
       </c>
       <c r="AH93" t="n">
@@ -13149,12 +13009,7 @@
           <t>You can reach me at student51@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG94" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG94" t="inlineStr"/>
       <c r="AH94" t="n">
         <v>99</v>
       </c>
@@ -13284,8 +13139,7 @@
       </c>
       <c r="AG95" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Feel free to reach out at abarnes@school.edu with any follow-up questions.</t>
         </is>
       </c>
       <c r="AH95" t="n">
@@ -13421,8 +13275,7 @@
       </c>
       <c r="AG96" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The "flipped classroom" approach didn't work for me.</t>
         </is>
       </c>
       <c r="AH96" t="n">
@@ -13554,8 +13407,7 @@
       </c>
       <c r="AG97" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I struggled with the pace at first, but it got better.</t>
         </is>
       </c>
       <c r="AH97" t="n">
@@ -13687,8 +13539,7 @@
       </c>
       <c r="AG98" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I really enjoyed working through proofs step by step.</t>
         </is>
       </c>
       <c r="AH98" t="n">
@@ -13820,8 +13671,7 @@
       </c>
       <c r="AG99" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The online videos were confusing, but the textbook helped.</t>
         </is>
       </c>
       <c r="AH99" t="n">
@@ -14084,12 +13934,7 @@
           <t>You can reach me at student16@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG101" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG101" t="inlineStr"/>
       <c r="AH101" t="n">
         <v>62</v>
       </c>
@@ -14223,8 +14068,7 @@
       </c>
       <c r="AG102" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH102" t="n">
@@ -14356,8 +14200,8 @@
       </c>
       <c r="AG103" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH103" t="n">
@@ -14489,8 +14333,8 @@
       </c>
       <c r="AG104" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>This was hard for me,
+but I learned a lot in the end.</t>
         </is>
       </c>
       <c r="AH104" t="n">
@@ -14622,8 +14466,7 @@
       </c>
       <c r="AG105" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Honestly, I think this was one of my favorite math classes.</t>
         </is>
       </c>
       <c r="AH105" t="n">
@@ -14755,8 +14598,7 @@
       </c>
       <c r="AG106" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH106" t="n">
@@ -14892,8 +14734,7 @@
       </c>
       <c r="AG107" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>More practice problems would help, please add some.</t>
         </is>
       </c>
       <c r="AH107" t="n">
@@ -15029,8 +14870,7 @@
       </c>
       <c r="AG108" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH108" t="n">
@@ -15166,8 +15006,7 @@
       </c>
       <c r="AG109" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I wish we had more time on word problems, graphs, and functions.</t>
         </is>
       </c>
       <c r="AH109" t="n">
@@ -15299,8 +15138,7 @@
       </c>
       <c r="AG110" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>I struggled with the pace at first, but it got better.</t>
         </is>
       </c>
       <c r="AH110" t="n">
@@ -15432,8 +15270,7 @@
       </c>
       <c r="AG111" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH111" t="n">
@@ -15565,8 +15402,7 @@
       </c>
       <c r="AG112" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Not enough feedback on homework, exams were tough, and grading was slow.</t>
         </is>
       </c>
       <c r="AH112" t="n">
@@ -15702,8 +15538,7 @@
       </c>
       <c r="AG113" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>The professor explained things clearly, and the TA was great too.</t>
         </is>
       </c>
       <c r="AH113" t="n">
@@ -15837,12 +15672,7 @@
           <t>You can reach me at student94@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG114" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG114" t="inlineStr"/>
       <c r="AH114" t="n">
         <v>63</v>
       </c>
@@ -15970,12 +15800,7 @@
           <t>You can reach me at student38@example.edu if you need more detail.</t>
         </is>
       </c>
-      <c r="AG115" t="inlineStr">
-        <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
-        </is>
-      </c>
+      <c r="AG115" t="inlineStr"/>
       <c r="AH115" t="n">
         <v>63</v>
       </c>
@@ -16105,8 +15930,7 @@
       </c>
       <c r="AG116" t="inlineStr">
         <is>
-          <t>I liked the pacing, the examples, and the "extra practice" set.
-Overall: solid, would recommend, 9/10.</t>
+          <t>Too much homework, not enough review before tests.</t>
         </is>
       </c>
       <c r="AH116" t="n">

</xml_diff>

<commit_message>
Practice data: real Q5 statements (Q5_4 negatively worded by meaning, not by a text marker); regenerate messy_qualtrics and survey.qsf
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MeiaEyWLPV5E9J6rB7YDUR
</commit_message>
<xml_diff>
--- a/fixtures/practice/messy_qualtrics/messy.xlsx
+++ b/fixtures/practice/messy_qualtrics/messy.xlsx
@@ -737,32 +737,32 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Matrix statement 1 about classroom experience</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - I enjoy coming to this class</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Matrix statement 2 about classroom experience</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - The teacher explains things clearly</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Matrix statement 3 about classroom experience</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - I feel comfortable asking questions</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Matrix statement 4 about classroom experience (reverse-worded)</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - I often feel lost in this class</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Matrix statement 5 about classroom experience</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - The activities help me learn</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Matrix statement 6 about classroom experience</t>
+          <t>Please say how much you agree with each statement about your classroom experience. - I would recommend this class to a friend</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">

</xml_diff>